<commit_message>
upd res & curve
</commit_message>
<xml_diff>
--- a/logs/scaleup/summary/oss_extrx_ce_std_analysis.xlsx
+++ b/logs/scaleup/summary/oss_extrx_ce_std_analysis.xlsx
@@ -555,7 +555,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=9; r=2</t>
+          <t>3/3 [##########]; s=8; r=1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -577,17 +577,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=15; r=3</t>
+          <t>3/3 [##########]; s=10; r=2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=8; r=1</t>
+          <t>3/3 [##########]; s=16; r=9</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=9; r=2</t>
+          <t>3/3 [##########]; s=12; r=3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=8; r=1</t>
+          <t>3/3 [##########]; s=12; r=2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=70; r=2</t>
+          <t>2/3 [#######---]; s=796.5; r=7.5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -636,12 +636,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=9; r=2</t>
+          <t>3/3 [##########]; s=8; r=1</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1/3 [###-------]; s=563; r=12</t>
+          <t>1/3 [###-------]; s=371; r=6</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -685,17 +685,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=8; r=1</t>
+          <t>3/3 [##########]; s=9; r=2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0/3 [----------]; s=NA; r=NA</t>
+          <t>1/3 [###-------]; s=509; r=9</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3/3 [##########]; s=599; r=9</t>
+          <t>1/3 [###-------]; s=793; r=9</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">

</xml_diff>